<commit_message>
refactor(sample): move tag label to sample data
</commit_message>
<xml_diff>
--- a/bioinformatics-analysis/resources/data-meta.xlsx
+++ b/bioinformatics-analysis/resources/data-meta.xlsx
@@ -1,124 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\20182\Desktop\项目\解读平台\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCF43AA8-3C24-4A56-A5E4-924CC341ED39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D889C858-21DA-46CE-AF41-06E67CB30F73}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>文库编号</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>捕获试剂盒</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>index类型</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>index编号</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>杂交input</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>核酸打断方式</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>送检机构</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>核酸类型</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>核酸降解等级</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>风险上机</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>样本识别号</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>R1文件</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>R2文件</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>建库input（ng）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>数据详情</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color rgb="FFFF0000"/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
       <sz val="9"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -134,31 +59,91 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -458,82 +443,120 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E592A456-6669-4BF8-849B-04997ACEBB3A}">
-  <dimension ref="A1:O1"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
-    <col min="3" max="3" width="10.4140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.4140625" bestFit="1" customWidth="1"/>
+    <col width="10.4140625" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" style="2" min="8" max="8"/>
+    <col width="10.4140625" bestFit="1" customWidth="1" style="2" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>12</v>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>数据详情</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>文库编号</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>捕获试剂盒</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>建库input（ng）</t>
+        </is>
+      </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>index类型</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>index编号</t>
+        </is>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>杂交input</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>核酸打断方式</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>送检机构</t>
+        </is>
+      </c>
+      <c r="J1" s="0" t="inlineStr">
+        <is>
+          <t>核酸类型</t>
+        </is>
+      </c>
+      <c r="K1" s="0" t="inlineStr">
+        <is>
+          <t>核酸降解等级</t>
+        </is>
+      </c>
+      <c r="L1" s="0" t="inlineStr">
+        <is>
+          <t>风险上机</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>样本识别号</t>
+        </is>
+      </c>
+      <c r="N1" s="0" t="inlineStr">
+        <is>
+          <t>Tag标签</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>R1文件</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>R2文件</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576" xr:uid="{745B25BD-335C-45D0-9D9F-14D894DE00AB}">
+    <dataValidation sqref="C2:C1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>"Exome Plus Panel v2.0,HiSNP Panel v1.0,HiSNP Ultra Panel v1.0,HLAtyping Panel v1.0,NanOnco Plus Panel v3.0,OncoFu Elite V1.0,Methlyation panel V1.0,LungCancer Panel v1.0,NanOnCT Panel v1.0"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576" xr:uid="{EFF00B2A-A17B-42A3-A29C-A41781D217B2}">
+    <dataValidation sqref="J2:J1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>"gDNA,cfDNA,RNA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K1048576" xr:uid="{DB35467D-72C1-4BBB-8332-8003F7497CA0}">
+    <dataValidation sqref="K2:K1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>"A,B,C,D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L1048576" xr:uid="{490BECAE-0A67-4F8D-8D48-3670505ED721}">
+    <dataValidation sqref="L2:L1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>"是,否"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{A88F6E40-7926-4393-A9A8-E576741E0327}">
+    <dataValidation sqref="D1:D1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="decimal">
       <formula1>0</formula1>
       <formula2>9999999999999</formula2>
     </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:G1048576" xr:uid="{C29D1A74-359D-4030-89A8-EB5C2D4ED9DE}">
+    <dataValidation sqref="G1:G1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="decimal">
       <formula1>0</formula1>
       <formula2>99999999999999</formula2>
     </dataValidation>

</xml_diff>